<commit_message>
Hide year color material fields and add quantity steppers across UI
</commit_message>
<xml_diff>
--- a/inventory-template.xlsx
+++ b/inventory-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:Q4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,42 +422,33 @@
         <v>scale</v>
       </c>
       <c r="H1" t="str">
-        <v>year</v>
+        <v>condition</v>
       </c>
       <c r="I1" t="str">
-        <v>color</v>
+        <v>mrp</v>
       </c>
       <c r="J1" t="str">
-        <v>material</v>
+        <v>price</v>
       </c>
       <c r="K1" t="str">
-        <v>condition</v>
+        <v>discount</v>
       </c>
       <c r="L1" t="str">
-        <v>mrp</v>
+        <v>quantity</v>
       </c>
       <c r="M1" t="str">
-        <v>price</v>
+        <v>isNew</v>
       </c>
       <c r="N1" t="str">
-        <v>discount</v>
+        <v>image</v>
       </c>
       <c r="O1" t="str">
-        <v>quantity</v>
+        <v>image2</v>
       </c>
       <c r="P1" t="str">
-        <v>isNew</v>
+        <v>image3</v>
       </c>
       <c r="Q1" t="str">
-        <v>image</v>
-      </c>
-      <c r="R1" t="str">
-        <v>image2</v>
-      </c>
-      <c r="S1" t="str">
-        <v>image3</v>
-      </c>
-      <c r="T1" t="str">
         <v>description</v>
       </c>
     </row>
@@ -484,39 +475,30 @@
         <v>1:64</v>
       </c>
       <c r="H2" t="str">
+        <v>Carded Mint</v>
+      </c>
+      <c r="I2" t="str">
         <v>1999</v>
       </c>
-      <c r="I2" t="str">
-        <v>Blue</v>
-      </c>
       <c r="J2" t="str">
-        <v>Diecast</v>
+        <v>1499</v>
       </c>
       <c r="K2" t="str">
-        <v>Carded Mint</v>
+        <v>25</v>
       </c>
       <c r="L2" t="str">
-        <v>1999</v>
+        <v>8</v>
       </c>
       <c r="M2" t="str">
-        <v>1499</v>
+        <v>TRUE</v>
       </c>
       <c r="N2" t="str">
-        <v>25</v>
+        <v>https://images.unsplash.com/photo-1619767886558-efdc259cde1a?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
       </c>
       <c r="O2" t="str">
-        <v>8</v>
-      </c>
-      <c r="P2" t="str">
-        <v>TRUE</v>
+        <v>https://images.unsplash.com/photo-1493238792000-8113da705763?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
       </c>
       <c r="Q2" t="str">
-        <v>https://images.unsplash.com/photo-1619767886558-efdc259cde1a?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
-      </c>
-      <c r="R2" t="str">
-        <v>https://images.unsplash.com/photo-1493238792000-8113da705763?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
-      </c>
-      <c r="T2" t="str">
         <v>JDM icon with collector-favorite casting.</v>
       </c>
     </row>
@@ -543,36 +525,27 @@
         <v>1:64</v>
       </c>
       <c r="H3" t="str">
-        <v>1998</v>
+        <v>Carded Good</v>
       </c>
       <c r="I3" t="str">
-        <v>Orange</v>
+        <v>899</v>
       </c>
       <c r="J3" t="str">
-        <v>Diecast</v>
+        <v>699</v>
       </c>
       <c r="K3" t="str">
-        <v>Carded Good</v>
+        <v>22</v>
       </c>
       <c r="L3" t="str">
-        <v>899</v>
+        <v>20</v>
       </c>
       <c r="M3" t="str">
-        <v>699</v>
+        <v>FALSE</v>
       </c>
       <c r="N3" t="str">
-        <v>22</v>
-      </c>
-      <c r="O3" t="str">
-        <v>20</v>
-      </c>
-      <c r="P3" t="str">
-        <v>FALSE</v>
+        <v>https://images.unsplash.com/photo-1493238792000-8113da705763?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
       </c>
       <c r="Q3" t="str">
-        <v>https://images.unsplash.com/photo-1493238792000-8113da705763?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
-      </c>
-      <c r="T3" t="str">
         <v>Mainline model suitable for bundle offers.</v>
       </c>
     </row>
@@ -599,45 +572,36 @@
         <v>1:64</v>
       </c>
       <c r="H4" t="str">
-        <v>2020</v>
+        <v>Carded Mint</v>
       </c>
       <c r="I4" t="str">
-        <v>Yellow</v>
+        <v>2399</v>
       </c>
       <c r="J4" t="str">
-        <v>Diecast</v>
+        <v>1999</v>
       </c>
       <c r="K4" t="str">
-        <v>Carded Mint</v>
+        <v>17</v>
       </c>
       <c r="L4" t="str">
-        <v>2399</v>
+        <v>5</v>
       </c>
       <c r="M4" t="str">
-        <v>1999</v>
+        <v>TRUE</v>
       </c>
       <c r="N4" t="str">
-        <v>17</v>
+        <v>https://images.unsplash.com/photo-1549399542-7e3f8b79c341?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
       </c>
       <c r="O4" t="str">
-        <v>5</v>
-      </c>
-      <c r="P4" t="str">
-        <v>TRUE</v>
+        <v>https://images.unsplash.com/photo-1580273916550-e323be2ae537?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
       </c>
       <c r="Q4" t="str">
-        <v>https://images.unsplash.com/photo-1549399542-7e3f8b79c341?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
-      </c>
-      <c r="R4" t="str">
-        <v>https://images.unsplash.com/photo-1580273916550-e323be2ae537?auto=format&amp;fit=crop&amp;w=900&amp;q=80</v>
-      </c>
-      <c r="T4" t="str">
         <v>Premium detailed model with strong demand.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>